<commit_message>
Adião de novos recursos
</commit_message>
<xml_diff>
--- a/DownloadTodosResultadosLoterias/downloads/DIA_DE_SORTE.xlsx
+++ b/DownloadTodosResultadosLoterias/downloads/DIA_DE_SORTE.xlsx
@@ -101310,6 +101310,83 @@
         <x:v/>
       </x:c>
     </x:row>
+    <x:row>
+      <x:c t="n">
+        <x:v>1309</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>28/09/2026</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>06</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>Maio</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v/>
+      </x:c>
+      <x:c t="str">
+        <x:v>R$0,00</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>R$3.623,40</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>1191</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>R$25,00</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>14815</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>R$5,00</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>46298</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>R$2,50</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>Sim</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>R$1.368.325,00</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>R$1.000.000,00</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v/>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:phoneticPr fontId="2" type="noConversion"/>
   <x:pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
@@ -101498,7 +101575,7 @@
   <documentManagement>
     <PublishingExpirationDate xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
     <PublishingStartDate xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <AtualizadoPeloTimerJobEm xmlns="4455b8ba-124f-46d5-aaaa-9813efd83d1e">2026-09-28T04:13:40+00:00</AtualizadoPeloTimerJobEm>
+    <AtualizadoPeloTimerJobEm xmlns="4455b8ba-124f-46d5-aaaa-9813efd83d1e">2026-09-29T04:11:43+00:00</AtualizadoPeloTimerJobEm>
   </documentManagement>
 </p:properties>
 </file>

</xml_diff>

<commit_message>
Adicionado a coluna Linha x Coluna  na rota linhas-dd-du
</commit_message>
<xml_diff>
--- a/DownloadTodosResultadosLoterias/downloads/DIA_DE_SORTE.xlsx
+++ b/DownloadTodosResultadosLoterias/downloads/DIA_DE_SORTE.xlsx
@@ -101387,6 +101387,160 @@
         <x:v/>
       </x:c>
     </x:row>
+    <x:row>
+      <x:c t="n">
+        <x:v>1310</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>29/09/2026</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>02</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>06</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>07</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>Abril</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v/>
+      </x:c>
+      <x:c t="str">
+        <x:v>R$0,00</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>R$2.603,98</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>1319</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>R$25,00</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>16569</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>R$5,00</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>61311</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>R$2,50</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>Sim</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>R$1.690.555,00</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>R$1.300.000,00</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v/>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c t="n">
+        <x:v>1311</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>01</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>02</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>08</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>09</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>Mar&amp;ccedil;o</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v/>
+      </x:c>
+      <x:c t="str">
+        <x:v>R$0,00</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>R$4.509,06</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>1272</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>R$25,00</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>17009</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>R$5,00</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>64423</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>R$2,50</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>Sim</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>R$1.713.360,00</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>R$1.500.000,00</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v/>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:phoneticPr fontId="2" type="noConversion"/>
   <x:pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
@@ -101575,7 +101729,7 @@
   <documentManagement>
     <PublishingExpirationDate xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
     <PublishingStartDate xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <AtualizadoPeloTimerJobEm xmlns="4455b8ba-124f-46d5-aaaa-9813efd83d1e">2026-09-29T04:11:43+00:00</AtualizadoPeloTimerJobEm>
+    <AtualizadoPeloTimerJobEm xmlns="4455b8ba-124f-46d5-aaaa-9813efd83d1e">2026-10-01T04:12:49+00:00</AtualizadoPeloTimerJobEm>
   </documentManagement>
 </p:properties>
 </file>

</xml_diff>

<commit_message>
Adiconado 'Análise detalhada das sequências'
</commit_message>
<xml_diff>
--- a/DownloadTodosResultadosLoterias/downloads/DIA_DE_SORTE.xlsx
+++ b/DownloadTodosResultadosLoterias/downloads/DIA_DE_SORTE.xlsx
@@ -101541,6 +101541,314 @@
         <x:v/>
       </x:c>
     </x:row>
+    <x:row>
+      <x:c t="n">
+        <x:v>1312</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>01/10/2026</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>02</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>08</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>Abril</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v/>
+      </x:c>
+      <x:c t="str">
+        <x:v>R$0,00</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>R$3.148,32</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>1919</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>R$25,00</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>22888</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>R$5,00</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>70419</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>R$2,50</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>Sim</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>R$2.108.130,00</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>R$1.800.000,00</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v/>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c t="n">
+        <x:v>1313</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>02/10/2026</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>07</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>Fevereiro</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v/>
+      </x:c>
+      <x:c t="str">
+        <x:v>R$0,00</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>R$2.736,42</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>1812</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>R$25,00</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>23753</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>R$5,00</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>71878</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>R$2,50</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>Sim</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>R$2.243.112,50</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>R$2.200.000,00</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v/>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c t="n">
+        <x:v>1314</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>03/10/2026</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>02</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>Junho</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v/>
+      </x:c>
+      <x:c t="str">
+        <x:v>R$0,00</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>76</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>R$1.998,66</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>2366</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>R$25,00</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>28391</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>R$5,00</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>76192</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>R$2,50</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>Sim</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>R$2.546.037,50</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>R$2.600.000,00</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v/>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c t="n">
+        <x:v>1315</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>05/10/2026</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>02</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>09</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>Outubro</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v/>
+      </x:c>
+      <x:c t="str">
+        <x:v>R$0,00</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>81</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>R$2.383,14</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>2549</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>R$25,00</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>29610</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>R$5,00</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>117806</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>R$2,50</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>Sim</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>R$2.625.575,00</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>R$2.900.000,00</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v/>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:phoneticPr fontId="2" type="noConversion"/>
   <x:pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
@@ -101729,7 +102037,7 @@
   <documentManagement>
     <PublishingExpirationDate xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
     <PublishingStartDate xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <AtualizadoPeloTimerJobEm xmlns="4455b8ba-124f-46d5-aaaa-9813efd83d1e">2026-10-01T04:12:49+00:00</AtualizadoPeloTimerJobEm>
+    <AtualizadoPeloTimerJobEm xmlns="4455b8ba-124f-46d5-aaaa-9813efd83d1e">2026-10-06T04:11:30+00:00</AtualizadoPeloTimerJobEm>
   </documentManagement>
 </p:properties>
 </file>

</xml_diff>

<commit_message>
Melhorias nos card da conferência
</commit_message>
<xml_diff>
--- a/DownloadTodosResultadosLoterias/downloads/DIA_DE_SORTE.xlsx
+++ b/DownloadTodosResultadosLoterias/downloads/DIA_DE_SORTE.xlsx
@@ -101849,6 +101849,314 @@
         <x:v/>
       </x:c>
     </x:row>
+    <x:row>
+      <x:c t="n">
+        <x:v>1316</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>06/10/2026</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>01</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>06</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>Setembro</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v/>
+      </x:c>
+      <x:c t="str">
+        <x:v>R$0,00</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>56</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>R$2.907,85</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>2482</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>R$25,00</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>30356</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>R$5,00</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>106294</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>R$2,50</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>Sim</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>R$2.865.930,00</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>R$3.300.000,00</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v/>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c t="n">
+        <x:v>1317</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>07/10/2026</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>04</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>07</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>Mar&amp;ccedil;o</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v/>
+      </x:c>
+      <x:c t="str">
+        <x:v>R$0,00</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>88</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>R$1.878,71</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>3182</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>R$25,00</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>36938</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>R$5,00</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>100114</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>R$2,50</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>Sim</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>R$2.972.810,00</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>R$3.700.000,00</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v/>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c t="n">
+        <x:v>1318</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>08/10/2026</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>01</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>02</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>03</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>Setembro</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v/>
+      </x:c>
+      <x:c t="str">
+        <x:v>R$0,00</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>R$3.656,52</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>2081</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>R$25,00</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>29357</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>R$5,00</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>109516</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>R$2,50</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>Sim</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>R$3.107.132,50</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>R$4.100.000,00</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v/>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c t="n">
+        <x:v>1319</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>09/10/2026</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>02</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>04</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>09</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>Janeiro</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>RIO DE JANEIRO/RJ</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>R$4.192.833,50</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>121</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>R$1.737,79</x:v>
+      </x:c>
+      <x:c t="n">
+        <x:v>3192</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>R$25,00</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>37082</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>R$5,00</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>96646</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>R$2,50</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>Não</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>R$3.443.987,50</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v>R$100.000,00</x:v>
+      </x:c>
+      <x:c t="str">
+        <x:v/>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:phoneticPr fontId="2" type="noConversion"/>
   <x:pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
@@ -102037,7 +102345,7 @@
   <documentManagement>
     <PublishingExpirationDate xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
     <PublishingStartDate xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <AtualizadoPeloTimerJobEm xmlns="4455b8ba-124f-46d5-aaaa-9813efd83d1e">2026-10-06T04:11:30+00:00</AtualizadoPeloTimerJobEm>
+    <AtualizadoPeloTimerJobEm xmlns="4455b8ba-124f-46d5-aaaa-9813efd83d1e">2026-10-11T04:11:57+00:00</AtualizadoPeloTimerJobEm>
   </documentManagement>
 </p:properties>
 </file>

</xml_diff>